<commit_message>
Corrida | ARG-COMD | 2026-06-17 11:53:35.410812
</commit_message>
<xml_diff>
--- a/indicadores/ARG-COMD_out.xlsx
+++ b/indicadores/ARG-COMD_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="513">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice de precios de materias primas de exportación (en USD)</t>
+    <t xml:space="preserve">Índice de precios de materias primas de exportación</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentina</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2049,9 +2055,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2062,7 +2072,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2076,7 +2086,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2092,7 +2102,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2120,7 +2130,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2134,7 +2144,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2162,7 +2172,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2176,7 +2186,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2190,7 +2200,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2204,7 +2214,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2220,7 +2230,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2234,7 +2244,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2382,10 +2392,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2398,10 +2408,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2425,66 +2435,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>121.94335403325</v>
@@ -2537,7 +2547,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>121.889312555128</v>
@@ -2594,7 +2604,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>123.922725895755</v>
@@ -2651,7 +2661,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>133.297527992546</v>
@@ -2708,7 +2718,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>132.62149251765</v>
@@ -2765,7 +2775,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>126.204128393042</v>
@@ -2822,7 +2832,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>125.322047354838</v>
@@ -2879,7 +2889,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>126.32700099826</v>
@@ -2936,7 +2946,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>125.211438278727</v>
@@ -2993,7 +3003,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>122.287442021719</v>
@@ -3050,7 +3060,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>119.80385326876</v>
@@ -3107,7 +3117,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>121.683832953038</v>
@@ -3164,7 +3174,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>154.6</v>
@@ -3223,7 +3233,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>150.8</v>
@@ -3282,7 +3292,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>153.3</v>
@@ -3341,7 +3351,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>149.9</v>
@@ -3400,7 +3410,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>149.3</v>
@@ -3459,7 +3469,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>138</v>
@@ -3518,7 +3528,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>134</v>
@@ -3577,7 +3587,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>139.2</v>
@@ -3636,7 +3646,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>139.6</v>
@@ -3695,7 +3705,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>144</v>
@@ -3754,7 +3764,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>145.6</v>
@@ -3813,7 +3823,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>137.5</v>
@@ -3872,7 +3882,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>128.6</v>
@@ -3931,7 +3941,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>124.6</v>
@@ -3990,7 +4000,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>118.7</v>
@@ -4049,7 +4059,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>114.5</v>
@@ -4108,7 +4118,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>115.2</v>
@@ -4167,7 +4177,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>107.9</v>
@@ -4226,7 +4236,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>106.1</v>
@@ -4285,7 +4295,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>99.9</v>
@@ -4344,7 +4354,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>102.2</v>
@@ -4403,7 +4413,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>105.6</v>
@@ -4462,7 +4472,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>105.6</v>
@@ -4521,7 +4531,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>102.2</v>
@@ -4580,7 +4590,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>100.7</v>
@@ -4639,7 +4649,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>94.7</v>
@@ -4698,7 +4708,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>96.1</v>
@@ -4757,7 +4767,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>98.4</v>
@@ -4816,7 +4826,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>97.3</v>
@@ -4875,7 +4885,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>96.5</v>
@@ -4934,7 +4944,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>96.6</v>
@@ -4993,7 +5003,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>103.2</v>
@@ -5052,7 +5062,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>107.6</v>
@@ -5111,7 +5121,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>106.7</v>
@@ -5170,7 +5180,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>107.3</v>
@@ -5229,7 +5239,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>107.3</v>
@@ -5288,7 +5298,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>110.1</v>
@@ -5347,7 +5357,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>113.2</v>
@@ -5406,7 +5416,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>112.1</v>
@@ -5465,7 +5475,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>107.4</v>
@@ -5524,7 +5534,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>113.8</v>
@@ -5583,7 +5593,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>113.1</v>
@@ -5642,7 +5652,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>108.9</v>
@@ -5701,7 +5711,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>109.5</v>
@@ -5760,7 +5770,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>116.1</v>
@@ -5819,7 +5829,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>115.8</v>
@@ -5878,7 +5888,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>119</v>
@@ -5937,7 +5947,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>115</v>
@@ -5996,7 +6006,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>114</v>
@@ -6055,7 +6065,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>110.8</v>
@@ -6114,7 +6124,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>106.2</v>
@@ -6173,7 +6183,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>105.3</v>
@@ -6232,7 +6242,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>109</v>
@@ -6291,7 +6301,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>109.2</v>
@@ -6350,7 +6360,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>110.1</v>
@@ -6409,7 +6419,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>111.3</v>
@@ -6468,7 +6478,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>109.4</v>
@@ -6527,7 +6537,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>101.9</v>
@@ -6586,7 +6596,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>101.2</v>
@@ -6645,7 +6655,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>100</v>
@@ -6704,7 +6714,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>100.395009575857</v>
@@ -6763,7 +6773,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>100.690581971988</v>
@@ -6822,7 +6832,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>106.421735100621</v>
@@ -6881,7 +6891,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>108.283467839848</v>
@@ -6940,7 +6950,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>110.651859639881</v>
@@ -6999,7 +7009,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>114.359158890613</v>
@@ -7058,7 +7068,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>121.922743006636</v>
@@ -7117,7 +7127,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>127.071089560406</v>
@@ -7176,7 +7186,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>129.179840249743</v>
@@ -7235,7 +7245,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>125.352073836389</v>
@@ -7294,7 +7304,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>122.396430238949</v>
@@ -7353,7 +7363,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>125.298314976386</v>
@@ -7412,7 +7422,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>128.387102797298</v>
@@ -7471,7 +7481,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>129.727113292119</v>
@@ -7530,7 +7540,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>128.347220547863</v>
@@ -7589,7 +7599,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>125.613557059402</v>
@@ -7648,7 +7658,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>129.775808729116</v>
@@ -7707,7 +7717,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>131.3268072954</v>
@@ -7766,7 +7776,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>130.56231520676</v>
@@ -7825,7 +7835,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>129.405136373491</v>
@@ -7884,7 +7894,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>135.805150352368</v>
@@ -7943,7 +7953,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>146.358441657937</v>
@@ -8002,7 +8012,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>152.215046608708</v>
@@ -8061,7 +8071,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>153.585588043796</v>
@@ -8120,7 +8130,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>161.449068618578</v>
@@ -8179,7 +8189,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>167.807290103546</v>
@@ -8238,7 +8248,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>183.684326850134</v>
@@ -8297,7 +8307,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>184.549316403564</v>
@@ -8356,7 +8366,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>181.897997421327</v>
@@ -8415,7 +8425,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>172.267141226526</v>
@@ -8474,7 +8484,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>170.303989857114</v>
@@ -8533,7 +8543,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>150.987531075223</v>
@@ -8592,7 +8602,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>143.6987482722</v>
@@ -8651,7 +8661,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>136.054915863852</v>
@@ -8710,7 +8720,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>133.002119827192</v>
@@ -8769,7 +8779,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>132.26097287608</v>
@@ -8828,7 +8838,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>134.697623824371</v>
@@ -8887,7 +8897,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>136.285707914467</v>
@@ -8946,7 +8956,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>148.906063980099</v>
@@ -9005,7 +9015,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>148.656739539305</v>
@@ -9064,7 +9074,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>148.196221569338</v>
@@ -9123,7 +9133,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>157.178430337039</v>
@@ -9182,7 +9192,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>157.741966731927</v>
@@ -9241,7 +9251,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>151.485640599832</v>
@@ -9300,7 +9310,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>144.473779230525</v>
@@ -9359,7 +9369,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>142.93785095608</v>
@@ -9418,7 +9428,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>142.176938284713</v>
@@ -9477,7 +9487,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>147.720602633648</v>
@@ -9536,7 +9546,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>151.386501750773</v>
@@ -9595,7 +9605,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>150.037451357623</v>
@@ -9654,7 +9664,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>150.949754185397</v>
@@ -9713,7 +9723,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>157.260093999224</v>
@@ -9772,7 +9782,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>163.846361369985</v>
@@ -9831,7 +9841,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>161.025115952535</v>
@@ -9890,7 +9900,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>163.979857071319</v>
@@ -9949,7 +9959,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>159.643178410891</v>
@@ -10008,7 +10018,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>159.15954804766</v>
@@ -10067,7 +10077,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>164.114369873103</v>
@@ -10126,7 +10136,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>172.632549206851</v>
@@ -10185,7 +10195,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>171.350625113422</v>
@@ -10244,7 +10254,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>168.941034368737</v>
@@ -10303,7 +10313,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>176.701782988876</v>
@@ -10362,7 +10372,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>182.650055988856</v>
@@ -10421,7 +10431,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>185.04669962955</v>
@@ -10480,7 +10490,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>191.228293928164</v>
@@ -10539,7 +10549,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>202.773662704957</v>
@@ -10598,7 +10608,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>205.809264863471</v>
@@ -10657,7 +10667,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>206.350586295294</v>
@@ -10716,7 +10726,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>222.219989124782</v>
@@ -10775,7 +10785,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>227.965817231756</v>
@@ -10834,7 +10844,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>245.302082906108</v>
@@ -10893,7 +10903,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>258.86662564083</v>
@@ -10952,7 +10962,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>278.092428253557</v>
@@ -11011,7 +11021,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>294.075767070782</v>
@@ -11070,7 +11080,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>289.930887674124</v>
@@ -11129,7 +11139,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>286.722455625919</v>
@@ -11188,7 +11198,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>290.850010365579</v>
@@ -11247,7 +11257,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>319.156266966409</v>
@@ -11306,7 +11316,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>324.40099016927</v>
@@ -11365,7 +11375,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>278.59904228172</v>
@@ -11424,7 +11434,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>257.900048921525</v>
@@ -11483,7 +11493,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>201.342888623244</v>
@@ -11542,7 +11552,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>188.701302639261</v>
@@ -11601,7 +11611,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>182.263358941971</v>
@@ -11660,7 +11670,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>199.946819970128</v>
@@ -11719,7 +11729,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>191.999275199393</v>
@@ -11778,7 +11788,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>191.292311657564</v>
@@ -11837,7 +11847,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>210.894101301514</v>
@@ -11896,7 +11906,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>232.391683087593</v>
@@ -11955,7 +11965,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>242.994213668503</v>
@@ -12014,7 +12024,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>219.328505323928</v>
@@ -12073,7 +12083,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>227.644126402256</v>
@@ -12132,7 +12142,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>217.62719983701</v>
@@ -12191,7 +12201,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>213.00687100768</v>
@@ -12250,7 +12260,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>221.039956387489</v>
@@ -12309,7 +12319,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>223.441605084719</v>
@@ -12368,7 +12378,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>219.439727847496</v>
@@ -12427,7 +12437,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>210.772601287601</v>
@@ -12486,7 +12496,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>210.55041094259</v>
@@ -12545,7 +12555,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>219.611075537924</v>
@@ -12604,7 +12614,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>215.51808842779</v>
@@ -12663,7 +12673,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>216.64823380128</v>
@@ -12722,7 +12732,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>226.067243091698</v>
@@ -12781,7 +12791,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>234.299309705643</v>
@@ -12840,7 +12850,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>238.297561484126</v>
@@ -12899,7 +12909,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>252.259804068191</v>
@@ -12958,7 +12968,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>269.041311051989</v>
@@ -13017,7 +13027,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>281.721175244922</v>
@@ -13076,7 +13086,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>295.88389993178</v>
@@ -13135,7 +13145,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>299.016118197328</v>
@@ -13194,7 +13204,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>297.760757073589</v>
@@ -13253,7 +13263,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>304.392142574678</v>
@@ -13312,7 +13322,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>300.802964753928</v>
@@ -13371,7 +13381,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>302.045843241147</v>
@@ -13430,7 +13440,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>302.041202333197</v>
@@ -13489,7 +13499,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>301.486597498986</v>
@@ -13548,7 +13558,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>295.2144104641</v>
@@ -13607,7 +13617,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>272.067370894796</v>
@@ -13666,7 +13676,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>268.15510912749</v>
@@ -13725,7 +13735,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>263.284032558957</v>
@@ -13784,7 +13794,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>276.411179968001</v>
@@ -13843,7 +13853,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>289.098404688058</v>
@@ -13902,7 +13912,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>303.078156432588</v>
@@ -13961,7 +13971,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>309.667295224539</v>
@@ -14020,7 +14030,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>305.722035329486</v>
@@ -14079,7 +14089,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>304.969373892139</v>
@@ -14138,7 +14148,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>341.393502083307</v>
@@ -14197,7 +14207,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>357.471871404646</v>
@@ -14256,7 +14266,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>353.959478251109</v>
@@ -14315,7 +14325,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>337.765971854844</v>
@@ -14374,7 +14384,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>326.5242771892</v>
@@ -14433,7 +14443,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>326.53593548068</v>
@@ -14492,7 +14502,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>321.76734980917</v>
@@ -14551,7 +14561,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>322.944231480406</v>
@@ -14610,7 +14620,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>317.689716290989</v>
@@ -14669,7 +14679,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>303.513014522052</v>
@@ -14728,7 +14738,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>312.81071574911</v>
@@ -14787,7 +14797,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>317.740607776332</v>
@@ -14846,7 +14856,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>317.767633242955</v>
@@ -14905,7 +14915,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>292.71011520124</v>
@@ -14964,7 +14974,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>295.252217277381</v>
@@ -15023,7 +15033,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>275.355228930007</v>
@@ -15082,7 +15092,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>273.200497131276</v>
@@ -15141,7 +15151,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>279.940908553031</v>
@@ -15200,7 +15210,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>274.125719856867</v>
@@ -15259,7 +15269,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>284.81943529804</v>
@@ -15318,7 +15328,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>291.776064485389</v>
@@ -15377,7 +15387,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>299.984959163076</v>
@@ -15436,7 +15446,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>298.99172120866</v>
@@ -15495,7 +15505,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>290.927948406536</v>
@@ -15554,7 +15564,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>268.906867049662</v>
@@ -15613,7 +15623,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>264.768492504345</v>
@@ -15672,7 +15682,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>265.929207253733</v>
@@ -15731,7 +15741,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>228.869194728345</v>
@@ -15790,7 +15800,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>248.629095504552</v>
@@ -15849,7 +15859,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>242.759941929508</v>
@@ -15908,7 +15918,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>225.283944639145</v>
@@ -15967,7 +15977,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>220.768322060654</v>
@@ -16026,7 +16036,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>216.777125778837</v>
@@ -16085,7 +16095,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>211.235441279401</v>
@@ -16144,7 +16154,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>208.738304708796</v>
@@ -16203,7 +16213,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>211.798287012352</v>
@@ -16262,7 +16272,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>221.896127030447</v>
@@ -16321,7 +16331,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>208.913234594631</v>
@@ -16380,7 +16390,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>198.041780142112</v>
@@ -16439,7 +16449,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>199.137543532265</v>
@@ -16498,7 +16508,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>190.45046176031</v>
@@ -16557,7 +16567,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>187.853397049479</v>
@@ -16616,7 +16626,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>183.742431421714</v>
@@ -16675,7 +16685,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>184.839168103619</v>
@@ -16734,7 +16744,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>188.677942504902</v>
@@ -16793,7 +16803,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>198.649832111227</v>
@@ -16852,7 +16862,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>217.265800818134</v>
@@ -16911,7 +16921,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>226.993416377508</v>
@@ -16970,7 +16980,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>212.171018142453</v>
@@ -17029,7 +17039,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>204.282647343349</v>
@@ -17088,7 +17098,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>201.866415054368</v>
@@ -17147,7 +17157,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>201.810170946885</v>
@@ -17206,7 +17216,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>203.374235173088</v>
@@ -17265,7 +17275,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>205.251539552478</v>
@@ -17324,7 +17334,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>208.61959613493</v>
@@ -17383,7 +17393,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>208.155143425737</v>
@@ -17442,7 +17452,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>203.268301733303</v>
@@ -17501,7 +17511,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>197.736607912316</v>
@@ -17560,7 +17570,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>200.119649270716</v>
@@ -17619,7 +17629,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>198.866728989128</v>
@@ -17678,7 +17688,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>204.33842410503</v>
@@ -17737,7 +17747,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>199.709434429971</v>
@@ -17796,7 +17806,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>202.167277351832</v>
@@ -17855,7 +17865,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>203.707053427394</v>
@@ -17914,7 +17924,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>203.919186043201</v>
@@ -17973,7 +17983,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>204.301454187787</v>
@@ -18032,7 +18042,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>210.094050354326</v>
@@ -18091,7 +18101,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>215.773100976693</v>
@@ -18150,7 +18160,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>221.561881186674</v>
@@ -18209,7 +18219,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>224.334311526471</v>
@@ -18268,7 +18278,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>226.949396575623</v>
@@ -18327,7 +18337,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>214.99732583762</v>
@@ -18386,7 +18396,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>207.133071240388</v>
@@ -18445,7 +18455,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>204.758594801175</v>
@@ -18504,7 +18514,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>199.993455175621</v>
@@ -18563,7 +18573,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>203.912844454551</v>
@@ -18622,7 +18632,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>200.986584818204</v>
@@ -18681,7 +18691,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>201.7174713017</v>
@@ -18740,7 +18750,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>204.584684902099</v>
@@ -18799,7 +18809,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>210.54134992609</v>
@@ -18858,7 +18868,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>204.082308832385</v>
@@ -18917,7 +18927,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>200.233507524888</v>
@@ -18976,7 +18986,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>199.939084938668</v>
@@ -19035,7 +19045,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>211.472311567281</v>
@@ -19094,7 +19104,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>209.310394132516</v>
@@ -19153,7 +19163,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>199.495242038024</v>
@@ -19212,7 +19222,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>200.66280512142</v>
@@ -19271,7 +19281,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>210.009903719707</v>
@@ -19330,7 +19340,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>207.202566255078</v>
@@ -19389,7 +19399,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>209.597146858909</v>
@@ -19448,7 +19458,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>214.207367324067</v>
@@ -19507,7 +19517,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>205.525503382835</v>
@@ -19566,7 +19576,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>193.54970654924</v>
@@ -19625,7 +19635,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>182.499675455443</v>
@@ -19684,7 +19694,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>182.608771197175</v>
@@ -19743,7 +19753,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>188.615357190677</v>
@@ -19802,7 +19812,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>194.665377580956</v>
@@ -19861,7 +19871,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>198.341980168309</v>
@@ -19920,7 +19930,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>210.241890933757</v>
@@ -19979,7 +19989,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>224.628510605522</v>
@@ -20038,7 +20048,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>237.742624501462</v>
@@ -20097,7 +20107,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>247.649280403626</v>
@@ -20156,7 +20166,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>270.878918358769</v>
@@ -20215,7 +20225,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>278.551730116435</v>
@@ -20274,7 +20284,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>281.561175584097</v>
@@ -20333,7 +20343,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>292.572783991031</v>
@@ -20392,7 +20402,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>317.612334775428</v>
@@ -20451,7 +20461,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>309.437129423979</v>
@@ -20510,7 +20520,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>295.806051167042</v>
@@ -20569,7 +20579,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>291.060245641188</v>
@@ -20628,7 +20638,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>277.018389261657</v>
@@ -20687,7 +20697,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>279.441346821957</v>
@@ -20746,7 +20756,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>289.866165836499</v>
@@ -20805,7 +20815,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>295.761824571776</v>
@@ -20864,7 +20874,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>310.638545937447</v>
@@ -20923,7 +20933,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>330.950896445181</v>
@@ -20982,7 +20992,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>367.716080219105</v>
@@ -21041,7 +21051,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>372.053751492309</v>
@@ -21100,7 +21110,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>372.810789908142</v>
@@ -21159,7 +21169,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>365.911036145177</v>
@@ -21218,7 +21228,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>338.174188680808</v>
@@ -21277,7 +21287,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>341.544477682754</v>
@@ -21336,7 +21346,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>331.991245166598</v>
@@ -21395,7 +21405,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>327.52756573524</v>
@@ -21454,7 +21464,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>330.720306963052</v>
@@ -21513,7 +21523,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>321.864711319773</v>
@@ -21572,7 +21582,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>328.331734902912</v>
@@ -21631,7 +21641,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>326.228888683105</v>
@@ -21690,7 +21700,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>314.067468077607</v>
@@ -21749,7 +21759,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>311.359891145018</v>
@@ -21808,7 +21818,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>292.10650844193</v>
@@ -21867,7 +21877,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>298.14986921858</v>
@@ -21926,7 +21936,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>308.338393855781</v>
@@ -21985,7 +21995,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>298.842715022802</v>
@@ -22044,7 +22054,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>291.624110716642</v>
@@ -22103,7 +22113,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>284.985211701701</v>
@@ -22162,7 +22172,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>287.625105319013</v>
@@ -22221,7 +22231,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>279.914278552095</v>
@@ -22280,7 +22290,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>267.949312983742</v>
@@ -22339,7 +22349,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>262.260744272657</v>
@@ -22398,7 +22408,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>261.709750679488</v>
@@ -22457,7 +22467,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>264.131666081208</v>
@@ -22516,7 +22526,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>270.885862375443</v>
@@ -22575,7 +22585,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>268.281140362254</v>
@@ -22634,7 +22644,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>262.569869518324</v>
@@ -22693,7 +22703,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>249.593499997287</v>
@@ -22752,7 +22762,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>250.081069162561</v>
@@ -22811,7 +22821,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>256.965597241146</v>
@@ -22870,7 +22880,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>249.724722467896</v>
@@ -22929,7 +22939,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>245.388777676865</v>
@@ -22988,7 +22998,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>255.134278551292</v>
@@ -23047,7 +23057,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>256.62085543464</v>
@@ -23106,7 +23116,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>248.85386187756</v>
@@ -23165,7 +23175,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>253.117072769163</v>
@@ -23224,7 +23234,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>251.095678221001</v>
@@ -23283,7 +23293,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>254.556712866669</v>
@@ -23342,7 +23352,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>251.791332225314</v>
@@ -23401,7 +23411,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>252.533306876165</v>
@@ -23460,7 +23470,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>259.021382768623</v>
@@ -23519,7 +23529,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>257.835602772269</v>
@@ -23578,7 +23588,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>264.012994223313</v>
@@ -23637,7 +23647,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>264.181777868084</v>
@@ -23696,7 +23706,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>265.936392367298</v>
@@ -23755,7 +23765,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>278.065767011568</v>
@@ -23814,7 +23824,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>305.359054853517</v>
@@ -23873,7 +23883,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>317.765871524664</v>
@@ -23932,7 +23942,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>321.370549005263</v>
@@ -23991,7 +24001,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3" t="n">
@@ -24024,7 +24034,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3" t="n">
@@ -24057,7 +24067,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3" t="n">
@@ -24090,7 +24100,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3" t="n">
@@ -24123,7 +24133,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3" t="n">
@@ -24156,7 +24166,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3" t="n">
@@ -24189,7 +24199,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3" t="n">
@@ -24222,7 +24232,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2"/>
       <c r="C374" s="3" t="n">
@@ -24255,7 +24265,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2"/>
       <c r="C375" s="3" t="n">
@@ -24288,7 +24298,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2"/>
       <c r="C376" s="3" t="n">
@@ -24321,7 +24331,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2"/>
       <c r="C377" s="3" t="n">
@@ -24354,7 +24364,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2"/>
       <c r="C378" s="3" t="n">
@@ -24387,7 +24397,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2"/>
       <c r="C379" s="3"/>
@@ -24410,7 +24420,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2"/>
       <c r="C380" s="3"/>
@@ -24433,7 +24443,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2"/>
       <c r="C381" s="3"/>
@@ -24456,7 +24466,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2"/>
       <c r="C382" s="3"/>
@@ -24479,7 +24489,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2"/>
       <c r="C383" s="3"/>
@@ -24502,7 +24512,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2"/>
       <c r="C384" s="3"/>
@@ -24525,7 +24535,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="3"/>
@@ -24548,7 +24558,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B386" s="2"/>
       <c r="C386" s="3"/>
@@ -24571,7 +24581,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B387" s="2"/>
       <c r="C387" s="3"/>
@@ -24594,7 +24604,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B388" s="2"/>
       <c r="C388" s="3"/>
@@ -24617,7 +24627,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B389" s="2"/>
       <c r="C389" s="3"/>
@@ -24640,7 +24650,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3"/>
@@ -24663,7 +24673,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3"/>
@@ -24686,7 +24696,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3"/>
@@ -24709,7 +24719,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3"/>
@@ -24732,7 +24742,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3"/>
@@ -24755,7 +24765,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3"/>
@@ -24778,7 +24788,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3"/>
@@ -24801,7 +24811,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3"/>
@@ -24824,7 +24834,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3"/>
@@ -24847,7 +24857,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3"/>
@@ -24870,7 +24880,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3"/>
@@ -24893,7 +24903,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3"/>
@@ -24916,7 +24926,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -24939,7 +24949,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -24962,7 +24972,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -24985,7 +24995,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25008,7 +25018,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25031,7 +25041,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25054,7 +25064,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25077,7 +25087,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25100,7 +25110,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25123,7 +25133,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -25146,7 +25156,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -25169,7 +25179,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -25192,7 +25202,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -25215,7 +25225,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -25238,7 +25248,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -25261,7 +25271,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -25284,7 +25294,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -25307,7 +25317,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -25330,7 +25340,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -25353,7 +25363,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -25387,97 +25397,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>
@@ -25501,7 +25511,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -25511,13 +25521,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.103450682511883</v>
@@ -25525,7 +25535,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.103179271666772</v>
@@ -25533,7 +25543,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.100251460942546</v>
@@ -25541,7 +25551,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.0988094082806618</v>
@@ -25549,7 +25559,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.093731900963494</v>
@@ -25557,7 +25567,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.105825671811418</v>
@@ -25565,7 +25575,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.142136225721984</v>
@@ -25573,7 +25583,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.19220259230448</v>
@@ -25581,7 +25591,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.239362322386611</v>
@@ -25589,7 +25599,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.268731384714011</v>
@@ -25597,7 +25607,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.258976152924555</v>
@@ -25605,7 +25615,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.211116926131424</v>
@@ -25613,7 +25623,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.161169046602974</v>
@@ -25621,7 +25631,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.120812214140729</v>
@@ -25629,7 +25639,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.0776911386446464</v>
@@ -25637,7 +25647,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.0394689819346639</v>
@@ -25645,7 +25655,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.0133227642214655</v>
@@ -25653,7 +25663,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.0140396527473733</v>
@@ -25661,7 +25671,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.0474654166681873</v>
@@ -25692,237 +25702,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{857BAB7D-5B28-4C21-9B87-1AE03CAB660A}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E39612ED-1BAC-46EB-9D72-7EC3710B7043}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED58D49C-79F7-4D7B-A324-C0CF5EFC528B}"/>
 </file>
</xml_diff>